<commit_message>
Add spreadsheet for JMatPro thermal Ti6Al4V prop.
</commit_message>
<xml_diff>
--- a/Temp_Properties/Temp_Properties_SI_Units.xlsx
+++ b/Temp_Properties/Temp_Properties_SI_Units.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mfree_iwf_ul_cut_refine_windows_ver\Temp_Properties\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{610106B6-2B33-4E1D-9C5B-976B3344F9BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79E65C0-707F-49AE-9950-AE95B2F435E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20520" yWindow="1830" windowWidth="20640" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3890,6 +3890,1884 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'SI_Units (2)'!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Poisson ratio (-)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="4"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SI_Units (2)'!$A$2:$A$100</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="99"/>
+                <c:pt idx="0">
+                  <c:v>298.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>303.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>313.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>323.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>333.15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>343.15</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>353.15</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>363.15</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>373.15</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>383.15</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>393.15</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>403.15</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>413.15</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>423.15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>433.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>443.15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>453.15</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>463.15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>473.15</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>483.15</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>493.15</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>503.15</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>513.15</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>523.15</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>533.15</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>543.15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>553.15</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>563.15</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>573.15</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>583.15</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>593.15</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>603.15</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>613.15</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>623.15</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>633.15</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>643.15</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>653.15</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>663.15</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>673.15</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>683.15</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>693.15</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>703.15</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>713.15</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>723.15</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>733.15</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>743.15</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>753.15</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>763.15</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>773.15</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>783.15</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>793.15</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>803.15</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>813.15</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>823.15</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>833.15</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>843.15</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>853.15</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>863.15</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>873.15</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>883.15</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>893.15</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>903.15</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>913.15</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>923.15</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>933.15</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>943.15</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>953.15</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>963.15</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>973.15</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>983.15</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>993.15</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>1003.15</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>1013.15</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>1023.15</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>1033.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>1043.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>1053.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>1063.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>1073.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>1083.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>1093.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>1103.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>1113.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>1123.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>1133.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>1143.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>1153.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>1163.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>1173.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>1183.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>1193.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>1203.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>1213.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>1223.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>1233.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>1243.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>1253.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>1263.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>1273.1500000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SI_Units (2)'!$F$2:$F$100</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="99"/>
+                <c:pt idx="0">
+                  <c:v>0.31797999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.31818000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.31857000000000002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.31896000000000002</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.31934000000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.31974000000000002</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.32013000000000003</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.32052000000000003</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.32090999999999997</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.32130999999999998</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.32169999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.3221</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.32249</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.32289000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.32329000000000002</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.32368999999999998</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.32408999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.32449</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.32489000000000001</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.32529999999999998</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.32569999999999999</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.3261</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.32651000000000002</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.32691999999999999</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.32732</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.32773000000000002</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.32813999999999999</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.32855000000000001</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.32895999999999997</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.32937</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.32978000000000002</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.33019999999999999</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.33061000000000001</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.33102999999999999</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.33144000000000001</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.33185999999999999</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.33228000000000002</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.3327</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.33312000000000003</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.33354</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.33395999999999998</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.33438000000000001</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.33479999999999999</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.33522999999999997</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.33565</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.33607999999999999</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.33650999999999998</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.33693000000000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.33735999999999999</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.33778999999999998</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.33822000000000002</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>0.33865000000000001</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>0.33907999999999999</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>0.33951999999999999</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>0.33994999999999997</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>0.34038000000000002</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>0.34082000000000001</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>0.34126000000000001</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>0.34168999999999999</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>0.34212999999999999</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>0.34256999999999999</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>0.34300999999999998</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>0.34344999999999998</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>0.34388999999999997</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>0.34433000000000002</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>0.34477999999999998</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>0.34522000000000003</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>0.34566999999999998</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>0.34610999999999997</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>0.34655999999999998</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>0.34700999999999999</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>0.34755999999999998</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>0.34814000000000001</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>0.34871999999999997</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>0.34932999999999997</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>0.34994999999999998</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>0.35060000000000002</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>0.35127000000000003</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>0.35197000000000001</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>0.35271000000000002</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>0.35348000000000002</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>0.3543</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>0.35515999999999998</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>0.35608000000000001</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>0.35705999999999999</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>0.35810999999999998</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>0.35922999999999999</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>0.36043999999999998</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>0.36174000000000001</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>0.36314999999999997</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>0.36465999999999998</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>0.36626999999999998</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>0.36797999999999997</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>0.36979000000000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>0.37165999999999999</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>0.37356</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>0.37546000000000002</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>0.37730999999999998</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>0.37902999999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3A02-4645-9403-2EFF7D882A73}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1187468432"/>
+        <c:axId val="1187460272"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1187468432"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1187460272"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1187460272"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1187468432"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'SI_Units (2)'!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Specific heat (J/(kg·K))</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="6"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SI_Units (2)'!$A$2:$A$100</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="99"/>
+                <c:pt idx="0">
+                  <c:v>298.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>303.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>313.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>323.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>333.15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>343.15</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>353.15</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>363.15</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>373.15</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>383.15</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>393.15</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>403.15</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>413.15</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>423.15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>433.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>443.15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>453.15</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>463.15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>473.15</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>483.15</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>493.15</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>503.15</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>513.15</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>523.15</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>533.15</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>543.15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>553.15</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>563.15</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>573.15</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>583.15</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>593.15</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>603.15</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>613.15</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>623.15</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>633.15</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>643.15</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>653.15</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>663.15</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>673.15</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>683.15</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>693.15</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>703.15</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>713.15</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>723.15</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>733.15</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>743.15</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>753.15</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>763.15</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>773.15</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>783.15</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>793.15</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>803.15</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>813.15</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>823.15</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>833.15</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>843.15</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>853.15</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>863.15</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>873.15</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>883.15</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>893.15</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>903.15</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>913.15</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>923.15</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>933.15</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>943.15</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>953.15</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>963.15</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>973.15</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>983.15</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>993.15</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>1003.15</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>1013.15</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>1023.15</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>1033.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>1043.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>1053.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>1063.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>1073.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>1083.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>1093.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>1103.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>1113.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>1123.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>1133.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>1143.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>1153.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>1163.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>1173.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>1183.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>1193.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>1203.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>1213.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>1223.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>1233.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>1243.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>1253.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>1263.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>1273.1500000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SI_Units (2)'!$G$2:$G$100</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="99"/>
+                <c:pt idx="0">
+                  <c:v>549.66999999999996</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>551.69000000000005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>555.57000000000005</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>559.26</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>562.79999999999995</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>566.18000000000006</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>569.43999999999994</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>572.57999999999993</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>575.62</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>578.57000000000005</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>581.43999999999994</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>584.23</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>586.94999999999993</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>589.62</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>592.21999999999991</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>594.78</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>597.29</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>599.76</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>602.19000000000005</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>604.58000000000004</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>606.94000000000005</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>609.27</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>611.58000000000004</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>613.86</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>616.11</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>618.34999999999991</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>620.55999999999995</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>622.75</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>624.92999999999995</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>627.09</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>629.24</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>631.37</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>633.49</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>635.6</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>637.68999999999994</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>639.78</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>641.85</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>643.92000000000007</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>645.97</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>648.0200000000001</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>650.05999999999995</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>652.1</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>654.1400000000001</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>656.19</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>658.25</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>660.32</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>662.39</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>664.4799999999999</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>666.57</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>668.68000000000006</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>670.79</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>672.92</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>675.06999999999994</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>677.22</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>679.38</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>681.56000000000006</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>683.75</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>685.94999999999993</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>688.17</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>690.39</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>692.63</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>694.85</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>697.25</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>699.68</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>702.13</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>703.42000000000007</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>704.73</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>706.09</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>707.5</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>708.94999999999993</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>763.73</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>769.59</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>776.22</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>783.73</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>792.23</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>801.84</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>812.71</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>824.85</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>838.73</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>854.40000000000009</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>872.09</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>892.02</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>913.34</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>938.25</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>964.9</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>995.53</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>1029</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>1064.8</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>1100.3800000000001</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>1138.3699999999999</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>1175.06</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>1205.6600000000001</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>1230.2</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>1241.4100000000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>1238.3599999999999</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>1217.1199999999999</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>1175.6400000000001</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>1117.26</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>1042.3399999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4C44-4473-B5EE-7C152CFF6841}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1242851904"/>
+        <c:axId val="1242851424"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1242851904"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1242851424"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1242851424"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1242851904"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -4011,6 +5889,86 @@
 </file>
 
 <file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -6114,20 +8072,1052 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>347807</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>85580</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>99</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>47048</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>161780</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6155,15 +9145,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>23812</xdr:rowOff>
+      <xdr:colOff>117186</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>124834</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>418522</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
+      <xdr:rowOff>13421</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6255,6 +9245,78 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>298738</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>119352</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>16741</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>7938</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C7B9C82-BE10-CF0C-FA28-F8405B6BFC22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>333374</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>129309</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>56283</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>58305</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC9C5192-88B8-FC13-2748-3017B262D79F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>

<commit_message>
feat(build): add OpenMP validation target and exclude test sources
- Add new `validate_omp` executable target for OpenMP benchmarking
- Exclude test source files (`src/tests/` and `test_omp_scaling.cpp`) from main application build
- Update Windows build instructions to exclude test directories
- Add project planning and todo documentation for OpenMP validation suite
- Include generated tool visualization files in results directory
</commit_message>
<xml_diff>
--- a/Temp_Properties/Temp_Properties_SI_Units.xlsx
+++ b/Temp_Properties/Temp_Properties_SI_Units.xlsx
@@ -5,24 +5,37 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mfree_iwf_ul_cut_refine_windows_ver\Temp_Properties\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gvwgroup-my.sharepoint.com/personal/gstyger_gvwholdings_com/Documents/Personal/mfree_iwf_ul_cut_refine_windows_ver/Temp_Properties/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79E65C0-707F-49AE-9950-AE95B2F435E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{C79E65C0-707F-49AE-9950-AE95B2F435E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BB4A74E-34D1-4117-BF0F-0AE628EF802C}"/>
   <bookViews>
-    <workbookView xWindow="-20520" yWindow="1830" windowWidth="20640" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="SI_Units" sheetId="2" r:id="rId2"/>
     <sheet name="SI_Units (2)" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
   <si>
     <t xml:space="preserve">T(K) </t>
   </si>
@@ -67,6 +80,12 @@
   </si>
   <si>
     <t>Specific heat (J/(kg·K))</t>
+  </si>
+  <si>
+    <t>rho_t</t>
+  </si>
+  <si>
+    <t>4459.647099-0.132016*T</t>
   </si>
 </sst>
 </file>
@@ -143,36 +162,6 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
@@ -884,6 +873,663 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-81D8-4911-95EB-736A1B1626BA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'SI_Units (2)'!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>rho_t</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SI_Units (2)'!$A$2:$A$100</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="99"/>
+                <c:pt idx="0">
+                  <c:v>298.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>303.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>313.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>323.14999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>333.15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>343.15</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>353.15</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>363.15</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>373.15</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>383.15</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>393.15</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>403.15</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>413.15</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>423.15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>433.15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>443.15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>453.15</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>463.15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>473.15</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>483.15</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>493.15</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>503.15</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>513.15</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>523.15</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>533.15</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>543.15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>553.15</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>563.15</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>573.15</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>583.15</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>593.15</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>603.15</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>613.15</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>623.15</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>633.15</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>643.15</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>653.15</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>663.15</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>673.15</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>683.15</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>693.15</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>703.15</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>713.15</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>723.15</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>733.15</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>743.15</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>753.15</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>763.15</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>773.15</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>783.15</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>793.15</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>803.15</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>813.15</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>823.15</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>833.15</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>843.15</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>853.15</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>863.15</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>873.15</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>883.15</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>893.15</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>903.15</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>913.15</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>923.15</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>933.15</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>943.15</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>953.15</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>963.15</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>973.15</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>983.15</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>993.15</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>1003.15</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>1013.15</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>1023.15</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>1033.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>1043.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>1053.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>1063.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>1073.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>1083.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>1093.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>1103.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>1113.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>1123.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>1133.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>1143.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>1153.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>1163.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>1173.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>1183.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>1193.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>1203.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>1213.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>1223.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>1233.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>1243.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>1253.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>1263.1500000000001</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>1273.1500000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SI_Units (2)'!$J$2:$J$100</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="99"/>
+                <c:pt idx="0">
+                  <c:v>4420.2865285999997</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4419.6264486</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4418.3062885999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4416.9861285999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4415.6659685999994</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4414.3458086000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4413.0256485999998</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4411.7054885999996</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4410.3853285999994</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4409.0651686000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4407.7450085999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4406.4248485999997</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4405.1046885999995</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4403.7845286000002</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4402.4643685999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4401.1442085999997</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4399.8240485999995</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4398.5038886000002</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4397.1837286</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4395.8635685999998</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>4394.5434085999996</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4393.2232485999994</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>4391.9030886</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>4390.5829285999998</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4389.2627685999996</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>4387.9426085999994</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>4386.6224486000001</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4385.3022885999999</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>4383.9821285999997</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>4382.6619685999995</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>4381.3418086000001</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>4380.0216485999999</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>4378.7014885999997</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>4377.3813285999995</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>4376.0611686000002</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>4374.7410086</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>4373.4208485999998</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>4372.1006885999996</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>4370.7805286000003</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>4369.4603686</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>4368.1402085999998</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>4366.8200485999996</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>4365.4998885999994</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>4364.1797286000001</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>4362.8595685999999</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>4361.5394085999997</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>4360.2192485999994</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>4358.8990886000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>4357.5789285999999</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>4356.2587685999997</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>4354.9386085999995</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>4353.6184486000002</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>4352.2982886</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>4350.9781285999998</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>4349.6579685999995</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>4348.3378086000002</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>4347.0176486</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>4345.6974885999998</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>4344.3773285999996</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>4343.0571685999994</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>4341.7370086000001</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>4340.4168485999999</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>4339.0966885999997</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>4337.7765285999994</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>4336.4563686000001</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>4335.1362085999999</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>4333.8160485999997</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>4332.4958885999995</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>4331.1757286000002</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>4329.8555686</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>4328.5354085999998</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>4327.2152485999995</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>4325.8950886000002</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>4324.5749286</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>4323.2547685999998</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>4321.9346085999996</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>4320.6144485999994</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>4319.2942886000001</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>4317.9741285999999</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>4316.6539685999996</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>4315.3338085999994</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>4314.0136486000001</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>4312.6934885999999</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>4311.3733285999997</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>4310.0531685999995</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>4308.7330086000002</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>4307.4128486</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>4306.0926885999997</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>4304.7725285999995</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>4303.4523686000002</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>4302.1322086</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>4300.8120485999998</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>4299.4918885999996</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>4298.1717285999994</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>4296.8515686000001</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>4295.5314085999998</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>4294.2112485999996</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>4292.8910885999994</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>4291.5709286000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-59C0-4A17-A17D-F46DDBB8F1BD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -9108,14 +9754,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>347807</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>492122</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>85580</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>47048</xdr:colOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>191363</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>161780</xdr:rowOff>
     </xdr:to>
@@ -9144,14 +9790,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>117186</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>261501</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>124834</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>418522</xdr:colOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>562837</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>13421</xdr:rowOff>
     </xdr:to>
@@ -9180,14 +9826,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>171450</xdr:colOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>315765</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>128587</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>14429</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>14287</xdr:rowOff>
     </xdr:to>
@@ -9216,14 +9862,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>325290</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>185737</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>485775</xdr:colOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>23954</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>71437</xdr:rowOff>
     </xdr:to>
@@ -9252,14 +9898,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>298738</xdr:colOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>443053</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>119352</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>16741</xdr:colOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>161056</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>7938</xdr:rowOff>
     </xdr:to>
@@ -9288,14 +9934,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>333374</xdr:colOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>477689</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>129309</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>56283</xdr:colOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>200598</xdr:colOff>
       <xdr:row>52</xdr:row>
       <xdr:rowOff>58305</xdr:rowOff>
     </xdr:to>
@@ -18098,7 +18744,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98DD581B-B0C6-4665-A929-DFD6D931C220}">
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -18110,7 +18756,7 @@
     <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -18132,8 +18778,14 @@
       <c r="G1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>298.14999999999998</v>
       </c>
@@ -18155,8 +18807,12 @@
       <c r="G2" s="2">
         <v>549.66999999999996</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J2">
+        <f>4459.647099-0.132016*A2</f>
+        <v>4420.2865285999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>303.14999999999998</v>
       </c>
@@ -18178,8 +18834,12 @@
       <c r="G3" s="2">
         <v>551.69000000000005</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J3">
+        <f t="shared" ref="J3:J66" si="0">4459.647099-0.132016*A3</f>
+        <v>4419.6264486</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>313.14999999999998</v>
       </c>
@@ -18201,8 +18861,12 @@
       <c r="G4" s="2">
         <v>555.57000000000005</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>4418.3062885999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>323.14999999999998</v>
       </c>
@@ -18224,8 +18888,12 @@
       <c r="G5" s="2">
         <v>559.26</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>4416.9861285999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>333.15</v>
       </c>
@@ -18247,8 +18915,12 @@
       <c r="G6" s="2">
         <v>562.79999999999995</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>4415.6659685999994</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>343.15</v>
       </c>
@@ -18270,8 +18942,12 @@
       <c r="G7" s="2">
         <v>566.18000000000006</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>4414.3458086000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>353.15</v>
       </c>
@@ -18293,8 +18969,12 @@
       <c r="G8" s="2">
         <v>569.43999999999994</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J8">
+        <f t="shared" si="0"/>
+        <v>4413.0256485999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>363.15</v>
       </c>
@@ -18316,8 +18996,12 @@
       <c r="G9" s="2">
         <v>572.57999999999993</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J9">
+        <f t="shared" si="0"/>
+        <v>4411.7054885999996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>373.15</v>
       </c>
@@ -18339,8 +19023,12 @@
       <c r="G10" s="2">
         <v>575.62</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J10">
+        <f t="shared" si="0"/>
+        <v>4410.3853285999994</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>383.15</v>
       </c>
@@ -18362,8 +19050,12 @@
       <c r="G11" s="2">
         <v>578.57000000000005</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>4409.0651686000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>393.15</v>
       </c>
@@ -18385,8 +19077,12 @@
       <c r="G12" s="2">
         <v>581.43999999999994</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J12">
+        <f t="shared" si="0"/>
+        <v>4407.7450085999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>403.15</v>
       </c>
@@ -18408,8 +19104,12 @@
       <c r="G13" s="2">
         <v>584.23</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>4406.4248485999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>413.15</v>
       </c>
@@ -18431,8 +19131,12 @@
       <c r="G14" s="2">
         <v>586.94999999999993</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J14">
+        <f t="shared" si="0"/>
+        <v>4405.1046885999995</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>423.15</v>
       </c>
@@ -18454,8 +19158,12 @@
       <c r="G15" s="2">
         <v>589.62</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J15">
+        <f t="shared" si="0"/>
+        <v>4403.7845286000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>433.15</v>
       </c>
@@ -18477,8 +19185,12 @@
       <c r="G16" s="2">
         <v>592.21999999999991</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J16">
+        <f t="shared" si="0"/>
+        <v>4402.4643685999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>443.15</v>
       </c>
@@ -18500,8 +19212,12 @@
       <c r="G17" s="2">
         <v>594.78</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J17">
+        <f t="shared" si="0"/>
+        <v>4401.1442085999997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>453.15</v>
       </c>
@@ -18523,8 +19239,12 @@
       <c r="G18" s="2">
         <v>597.29</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J18">
+        <f t="shared" si="0"/>
+        <v>4399.8240485999995</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>463.15</v>
       </c>
@@ -18546,8 +19266,12 @@
       <c r="G19" s="2">
         <v>599.76</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J19">
+        <f t="shared" si="0"/>
+        <v>4398.5038886000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>473.15</v>
       </c>
@@ -18569,8 +19293,12 @@
       <c r="G20" s="2">
         <v>602.19000000000005</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J20">
+        <f t="shared" si="0"/>
+        <v>4397.1837286</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>483.15</v>
       </c>
@@ -18592,8 +19320,12 @@
       <c r="G21" s="2">
         <v>604.58000000000004</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J21">
+        <f t="shared" si="0"/>
+        <v>4395.8635685999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>493.15</v>
       </c>
@@ -18615,8 +19347,12 @@
       <c r="G22" s="2">
         <v>606.94000000000005</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J22">
+        <f t="shared" si="0"/>
+        <v>4394.5434085999996</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>503.15</v>
       </c>
@@ -18638,8 +19374,12 @@
       <c r="G23" s="2">
         <v>609.27</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J23">
+        <f t="shared" si="0"/>
+        <v>4393.2232485999994</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>513.15</v>
       </c>
@@ -18661,8 +19401,12 @@
       <c r="G24" s="2">
         <v>611.58000000000004</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J24">
+        <f t="shared" si="0"/>
+        <v>4391.9030886</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>523.15</v>
       </c>
@@ -18684,8 +19428,12 @@
       <c r="G25" s="2">
         <v>613.86</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J25">
+        <f t="shared" si="0"/>
+        <v>4390.5829285999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>533.15</v>
       </c>
@@ -18707,8 +19455,12 @@
       <c r="G26" s="2">
         <v>616.11</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J26">
+        <f t="shared" si="0"/>
+        <v>4389.2627685999996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>543.15</v>
       </c>
@@ -18730,8 +19482,12 @@
       <c r="G27" s="2">
         <v>618.34999999999991</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J27">
+        <f t="shared" si="0"/>
+        <v>4387.9426085999994</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>553.15</v>
       </c>
@@ -18753,8 +19509,12 @@
       <c r="G28" s="2">
         <v>620.55999999999995</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J28">
+        <f t="shared" si="0"/>
+        <v>4386.6224486000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>563.15</v>
       </c>
@@ -18776,8 +19536,12 @@
       <c r="G29" s="2">
         <v>622.75</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J29">
+        <f t="shared" si="0"/>
+        <v>4385.3022885999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>573.15</v>
       </c>
@@ -18799,8 +19563,12 @@
       <c r="G30" s="2">
         <v>624.92999999999995</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J30">
+        <f t="shared" si="0"/>
+        <v>4383.9821285999997</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>583.15</v>
       </c>
@@ -18822,8 +19590,12 @@
       <c r="G31" s="2">
         <v>627.09</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J31">
+        <f t="shared" si="0"/>
+        <v>4382.6619685999995</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>593.15</v>
       </c>
@@ -18845,8 +19617,12 @@
       <c r="G32" s="2">
         <v>629.24</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J32">
+        <f t="shared" si="0"/>
+        <v>4381.3418086000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>603.15</v>
       </c>
@@ -18868,8 +19644,12 @@
       <c r="G33" s="2">
         <v>631.37</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J33">
+        <f t="shared" si="0"/>
+        <v>4380.0216485999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>613.15</v>
       </c>
@@ -18891,8 +19671,12 @@
       <c r="G34" s="2">
         <v>633.49</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J34">
+        <f t="shared" si="0"/>
+        <v>4378.7014885999997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>623.15</v>
       </c>
@@ -18914,8 +19698,12 @@
       <c r="G35" s="2">
         <v>635.6</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J35">
+        <f t="shared" si="0"/>
+        <v>4377.3813285999995</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>633.15</v>
       </c>
@@ -18937,8 +19725,12 @@
       <c r="G36" s="2">
         <v>637.68999999999994</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J36">
+        <f t="shared" si="0"/>
+        <v>4376.0611686000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>643.15</v>
       </c>
@@ -18960,8 +19752,12 @@
       <c r="G37" s="2">
         <v>639.78</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J37">
+        <f t="shared" si="0"/>
+        <v>4374.7410086</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>653.15</v>
       </c>
@@ -18983,8 +19779,12 @@
       <c r="G38" s="2">
         <v>641.85</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J38">
+        <f t="shared" si="0"/>
+        <v>4373.4208485999998</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>663.15</v>
       </c>
@@ -19006,8 +19806,12 @@
       <c r="G39" s="2">
         <v>643.92000000000007</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J39">
+        <f t="shared" si="0"/>
+        <v>4372.1006885999996</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>673.15</v>
       </c>
@@ -19029,8 +19833,12 @@
       <c r="G40" s="2">
         <v>645.97</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J40">
+        <f t="shared" si="0"/>
+        <v>4370.7805286000003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>683.15</v>
       </c>
@@ -19052,8 +19860,12 @@
       <c r="G41" s="2">
         <v>648.0200000000001</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J41">
+        <f t="shared" si="0"/>
+        <v>4369.4603686</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>693.15</v>
       </c>
@@ -19075,8 +19887,12 @@
       <c r="G42" s="2">
         <v>650.05999999999995</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J42">
+        <f t="shared" si="0"/>
+        <v>4368.1402085999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>703.15</v>
       </c>
@@ -19098,8 +19914,12 @@
       <c r="G43" s="2">
         <v>652.1</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J43">
+        <f t="shared" si="0"/>
+        <v>4366.8200485999996</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>713.15</v>
       </c>
@@ -19121,8 +19941,12 @@
       <c r="G44" s="2">
         <v>654.1400000000001</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J44">
+        <f t="shared" si="0"/>
+        <v>4365.4998885999994</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>723.15</v>
       </c>
@@ -19144,8 +19968,12 @@
       <c r="G45" s="2">
         <v>656.19</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J45">
+        <f t="shared" si="0"/>
+        <v>4364.1797286000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>733.15</v>
       </c>
@@ -19167,8 +19995,12 @@
       <c r="G46" s="2">
         <v>658.25</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J46">
+        <f t="shared" si="0"/>
+        <v>4362.8595685999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>743.15</v>
       </c>
@@ -19190,8 +20022,12 @@
       <c r="G47" s="2">
         <v>660.32</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J47">
+        <f t="shared" si="0"/>
+        <v>4361.5394085999997</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>753.15</v>
       </c>
@@ -19213,8 +20049,12 @@
       <c r="G48" s="2">
         <v>662.39</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J48">
+        <f t="shared" si="0"/>
+        <v>4360.2192485999994</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>763.15</v>
       </c>
@@ -19236,8 +20076,12 @@
       <c r="G49" s="2">
         <v>664.4799999999999</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J49">
+        <f t="shared" si="0"/>
+        <v>4358.8990886000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>773.15</v>
       </c>
@@ -19259,8 +20103,12 @@
       <c r="G50" s="2">
         <v>666.57</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J50">
+        <f t="shared" si="0"/>
+        <v>4357.5789285999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>783.15</v>
       </c>
@@ -19282,8 +20130,12 @@
       <c r="G51" s="2">
         <v>668.68000000000006</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J51">
+        <f t="shared" si="0"/>
+        <v>4356.2587685999997</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>793.15</v>
       </c>
@@ -19305,8 +20157,12 @@
       <c r="G52" s="2">
         <v>670.79</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J52">
+        <f t="shared" si="0"/>
+        <v>4354.9386085999995</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>803.15</v>
       </c>
@@ -19328,8 +20184,12 @@
       <c r="G53" s="2">
         <v>672.92</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J53">
+        <f t="shared" si="0"/>
+        <v>4353.6184486000002</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>813.15</v>
       </c>
@@ -19351,8 +20211,12 @@
       <c r="G54" s="2">
         <v>675.06999999999994</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J54">
+        <f t="shared" si="0"/>
+        <v>4352.2982886</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>823.15</v>
       </c>
@@ -19374,8 +20238,12 @@
       <c r="G55" s="2">
         <v>677.22</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J55">
+        <f t="shared" si="0"/>
+        <v>4350.9781285999998</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>833.15</v>
       </c>
@@ -19397,8 +20265,12 @@
       <c r="G56" s="2">
         <v>679.38</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J56">
+        <f t="shared" si="0"/>
+        <v>4349.6579685999995</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>843.15</v>
       </c>
@@ -19420,8 +20292,12 @@
       <c r="G57" s="2">
         <v>681.56000000000006</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J57">
+        <f t="shared" si="0"/>
+        <v>4348.3378086000002</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>853.15</v>
       </c>
@@ -19443,8 +20319,12 @@
       <c r="G58" s="2">
         <v>683.75</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J58">
+        <f t="shared" si="0"/>
+        <v>4347.0176486</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>863.15</v>
       </c>
@@ -19466,8 +20346,12 @@
       <c r="G59" s="2">
         <v>685.94999999999993</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J59">
+        <f t="shared" si="0"/>
+        <v>4345.6974885999998</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>873.15</v>
       </c>
@@ -19489,8 +20373,12 @@
       <c r="G60" s="2">
         <v>688.17</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J60">
+        <f t="shared" si="0"/>
+        <v>4344.3773285999996</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>883.15</v>
       </c>
@@ -19512,8 +20400,12 @@
       <c r="G61" s="2">
         <v>690.39</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J61">
+        <f t="shared" si="0"/>
+        <v>4343.0571685999994</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>893.15</v>
       </c>
@@ -19535,8 +20427,12 @@
       <c r="G62" s="2">
         <v>692.63</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J62">
+        <f t="shared" si="0"/>
+        <v>4341.7370086000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>903.15</v>
       </c>
@@ -19558,8 +20454,12 @@
       <c r="G63" s="2">
         <v>694.85</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J63">
+        <f t="shared" si="0"/>
+        <v>4340.4168485999999</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>913.15</v>
       </c>
@@ -19581,8 +20481,12 @@
       <c r="G64" s="2">
         <v>697.25</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J64">
+        <f t="shared" si="0"/>
+        <v>4339.0966885999997</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>923.15</v>
       </c>
@@ -19604,8 +20508,12 @@
       <c r="G65" s="2">
         <v>699.68</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J65">
+        <f t="shared" si="0"/>
+        <v>4337.7765285999994</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>933.15</v>
       </c>
@@ -19627,8 +20535,12 @@
       <c r="G66" s="2">
         <v>702.13</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J66">
+        <f t="shared" si="0"/>
+        <v>4336.4563686000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>943.15</v>
       </c>
@@ -19650,8 +20562,12 @@
       <c r="G67" s="2">
         <v>703.42000000000007</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J67">
+        <f t="shared" ref="J67:J100" si="1">4459.647099-0.132016*A67</f>
+        <v>4335.1362085999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>953.15</v>
       </c>
@@ -19673,8 +20589,12 @@
       <c r="G68" s="2">
         <v>704.73</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J68">
+        <f t="shared" si="1"/>
+        <v>4333.8160485999997</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>963.15</v>
       </c>
@@ -19696,8 +20616,12 @@
       <c r="G69" s="2">
         <v>706.09</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J69">
+        <f t="shared" si="1"/>
+        <v>4332.4958885999995</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>973.15</v>
       </c>
@@ -19719,8 +20643,12 @@
       <c r="G70" s="2">
         <v>707.5</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J70">
+        <f t="shared" si="1"/>
+        <v>4331.1757286000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>983.15</v>
       </c>
@@ -19742,8 +20670,12 @@
       <c r="G71" s="2">
         <v>708.94999999999993</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J71">
+        <f t="shared" si="1"/>
+        <v>4329.8555686</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>993.15</v>
       </c>
@@ -19765,8 +20697,12 @@
       <c r="G72" s="2">
         <v>763.73</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J72">
+        <f t="shared" si="1"/>
+        <v>4328.5354085999998</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>1003.15</v>
       </c>
@@ -19788,8 +20724,12 @@
       <c r="G73" s="2">
         <v>769.59</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J73">
+        <f t="shared" si="1"/>
+        <v>4327.2152485999995</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>1013.15</v>
       </c>
@@ -19811,8 +20751,12 @@
       <c r="G74" s="2">
         <v>776.22</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J74">
+        <f t="shared" si="1"/>
+        <v>4325.8950886000002</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>1023.15</v>
       </c>
@@ -19834,8 +20778,12 @@
       <c r="G75" s="2">
         <v>783.73</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J75">
+        <f t="shared" si="1"/>
+        <v>4324.5749286</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>1033.1500000000001</v>
       </c>
@@ -19857,8 +20805,12 @@
       <c r="G76" s="2">
         <v>792.23</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J76">
+        <f t="shared" si="1"/>
+        <v>4323.2547685999998</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>1043.1500000000001</v>
       </c>
@@ -19880,8 +20832,12 @@
       <c r="G77" s="2">
         <v>801.84</v>
       </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J77">
+        <f t="shared" si="1"/>
+        <v>4321.9346085999996</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>1053.1500000000001</v>
       </c>
@@ -19903,8 +20859,12 @@
       <c r="G78" s="2">
         <v>812.71</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J78">
+        <f t="shared" si="1"/>
+        <v>4320.6144485999994</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>1063.1500000000001</v>
       </c>
@@ -19926,8 +20886,12 @@
       <c r="G79" s="2">
         <v>824.85</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J79">
+        <f t="shared" si="1"/>
+        <v>4319.2942886000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>1073.1500000000001</v>
       </c>
@@ -19949,8 +20913,12 @@
       <c r="G80" s="2">
         <v>838.73</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J80">
+        <f t="shared" si="1"/>
+        <v>4317.9741285999999</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>1083.1500000000001</v>
       </c>
@@ -19972,8 +20940,12 @@
       <c r="G81" s="2">
         <v>854.40000000000009</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J81">
+        <f t="shared" si="1"/>
+        <v>4316.6539685999996</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>1093.1500000000001</v>
       </c>
@@ -19995,8 +20967,12 @@
       <c r="G82" s="2">
         <v>872.09</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J82">
+        <f t="shared" si="1"/>
+        <v>4315.3338085999994</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>1103.1500000000001</v>
       </c>
@@ -20018,8 +20994,12 @@
       <c r="G83" s="2">
         <v>892.02</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J83">
+        <f t="shared" si="1"/>
+        <v>4314.0136486000001</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>1113.1500000000001</v>
       </c>
@@ -20041,8 +21021,12 @@
       <c r="G84" s="2">
         <v>913.34</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J84">
+        <f t="shared" si="1"/>
+        <v>4312.6934885999999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>1123.1500000000001</v>
       </c>
@@ -20064,8 +21048,12 @@
       <c r="G85" s="2">
         <v>938.25</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J85">
+        <f t="shared" si="1"/>
+        <v>4311.3733285999997</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>1133.1500000000001</v>
       </c>
@@ -20087,8 +21075,12 @@
       <c r="G86" s="2">
         <v>964.9</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J86">
+        <f t="shared" si="1"/>
+        <v>4310.0531685999995</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>1143.1500000000001</v>
       </c>
@@ -20110,8 +21102,12 @@
       <c r="G87" s="2">
         <v>995.53</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J87">
+        <f t="shared" si="1"/>
+        <v>4308.7330086000002</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>1153.1500000000001</v>
       </c>
@@ -20133,8 +21129,12 @@
       <c r="G88" s="2">
         <v>1029</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J88">
+        <f t="shared" si="1"/>
+        <v>4307.4128486</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>1163.1500000000001</v>
       </c>
@@ -20156,8 +21156,12 @@
       <c r="G89" s="2">
         <v>1064.8</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J89">
+        <f t="shared" si="1"/>
+        <v>4306.0926885999997</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>1173.1500000000001</v>
       </c>
@@ -20179,8 +21183,12 @@
       <c r="G90" s="2">
         <v>1100.3800000000001</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J90">
+        <f t="shared" si="1"/>
+        <v>4304.7725285999995</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>1183.1500000000001</v>
       </c>
@@ -20202,8 +21210,12 @@
       <c r="G91" s="2">
         <v>1138.3699999999999</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J91">
+        <f t="shared" si="1"/>
+        <v>4303.4523686000002</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>1193.1500000000001</v>
       </c>
@@ -20225,8 +21237,12 @@
       <c r="G92" s="2">
         <v>1175.06</v>
       </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J92">
+        <f t="shared" si="1"/>
+        <v>4302.1322086</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>1203.1500000000001</v>
       </c>
@@ -20248,8 +21264,12 @@
       <c r="G93" s="2">
         <v>1205.6600000000001</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J93">
+        <f t="shared" si="1"/>
+        <v>4300.8120485999998</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>1213.1500000000001</v>
       </c>
@@ -20271,8 +21291,12 @@
       <c r="G94" s="2">
         <v>1230.2</v>
       </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J94">
+        <f t="shared" si="1"/>
+        <v>4299.4918885999996</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>1223.1500000000001</v>
       </c>
@@ -20294,8 +21318,12 @@
       <c r="G95" s="2">
         <v>1241.4100000000001</v>
       </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J95">
+        <f t="shared" si="1"/>
+        <v>4298.1717285999994</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>1233.1500000000001</v>
       </c>
@@ -20317,8 +21345,12 @@
       <c r="G96" s="2">
         <v>1238.3599999999999</v>
       </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J96">
+        <f t="shared" si="1"/>
+        <v>4296.8515686000001</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>1243.1500000000001</v>
       </c>
@@ -20340,8 +21372,12 @@
       <c r="G97" s="2">
         <v>1217.1199999999999</v>
       </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J97">
+        <f t="shared" si="1"/>
+        <v>4295.5314085999998</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>1253.1500000000001</v>
       </c>
@@ -20363,8 +21399,12 @@
       <c r="G98" s="2">
         <v>1175.6400000000001</v>
       </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J98">
+        <f t="shared" si="1"/>
+        <v>4294.2112485999996</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>1263.1500000000001</v>
       </c>
@@ -20386,8 +21426,12 @@
       <c r="G99" s="2">
         <v>1117.26</v>
       </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J99">
+        <f t="shared" si="1"/>
+        <v>4292.8910885999994</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>1273.1500000000001</v>
       </c>
@@ -20408,6 +21452,10 @@
       </c>
       <c r="G100" s="2">
         <v>1042.3399999999999</v>
+      </c>
+      <c r="J100">
+        <f t="shared" si="1"/>
+        <v>4291.5709286000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Temp_Properties SI units spreadsheet
Replace Temp_Properties/Temp_Properties_SI_Units.xlsx with an updated Excel file containing revised temperature property data in SI units. This is a binary change so detailed diffs are not shown in the git output.
</commit_message>
<xml_diff>
--- a/Temp_Properties/Temp_Properties_SI_Units.xlsx
+++ b/Temp_Properties/Temp_Properties_SI_Units.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mfree_iwf_ul_cut_refine_windows_ver\Temp_Properties\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D5C556-1F62-457D-A4FD-B128E748CC4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7BA40D-473E-43ED-B118-B28436B9B791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20520" yWindow="1830" windowWidth="20640" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20272,16 +20272,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>492122</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>196847</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>85580</xdr:rowOff>
+      <xdr:rowOff>57005</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>191363</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>505688</xdr:colOff>
       <xdr:row>50</xdr:row>
-      <xdr:rowOff>161780</xdr:rowOff>
+      <xdr:rowOff>133205</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -20310,14 +20310,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>261501</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>90051</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>124834</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>562837</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>391387</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>13421</xdr:rowOff>
     </xdr:to>
@@ -20348,16 +20348,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>315765</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>128587</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>553890</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>138112</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>14429</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>14287</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>252554</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -20386,14 +20386,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>325290</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>153840</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>185737</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>23954</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>462104</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>71437</xdr:rowOff>
     </xdr:to>
@@ -20424,16 +20424,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>443053</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>119352</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>585928</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>166977</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>161056</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>7938</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>303931</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>55563</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -20462,16 +20462,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>477689</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>129309</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>591989</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>62634</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>200598</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>58305</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>314898</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>182130</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>